<commit_message>
refactor: Update Excel formatting and calculations in excel_processor.py
</commit_message>
<xml_diff>
--- a/Dashboards/Dashboardv4.xlsx
+++ b/Dashboards/Dashboardv4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\CGC\Dashboards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB41EC3-8225-4E88-9215-4BBAC9A3A6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465BE206-F3C8-4504-B934-B06D4E490FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{84E4215D-59A1-47B3-B7C6-EBA92DED9849}"/>
   </bookViews>
@@ -72,23 +72,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -98,24 +84,46 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -230,57 +238,58 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -630,125 +639,127 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="30.140625" defaultRowHeight="42" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" style="3"/>
+    <col min="3" max="3" width="30.140625" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="30.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="10" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="H1" s="5"/>
+      <c r="F1" s="2"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="8">
+      <c r="D2" s="8"/>
+      <c r="E2" s="9">
         <f>IF(C3*0.2&lt;0,0,C3*0.2)</f>
         <v>4000</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="H2" s="4"/>
+      <c r="F2" s="9"/>
+      <c r="H2" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+      <c r="A3" s="11">
         <v>80000</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="11">
         <v>60000</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <f>A3-B3</f>
         <v>20000</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="10" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10"/>
+      <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="8">
+      <c r="D5" s="15"/>
+      <c r="E5" s="9">
         <f>IF(C6&lt;=125000,0,(C6-125000)*0.125)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="8"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
+      <c r="A6" s="11">
         <v>650000</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="11">
         <v>700000</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16">
         <f>A6-B6</f>
         <v>-50000</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="8">
+      <c r="B7" s="17"/>
+      <c r="C7" s="9">
         <f>SUM(E2,E5)</f>
         <v>4000</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8">
+      <c r="B8" s="18"/>
+      <c r="C8" s="18">
         <f>C3+C6</f>
         <v>-30000</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
fix(ExcelProcessor): Replace ROUNDDOWN with ROUND for tax calculations and improve formatting in `Capital Gains Data` worksheet
**The Latest changes made to `Capital Gains` worksheet can be seen in `Dashboards/Dashboardv4.xlsx`**
</commit_message>
<xml_diff>
--- a/Dashboards/Dashboardv4.xlsx
+++ b/Dashboards/Dashboardv4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\CGC\Dashboards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465BE206-F3C8-4504-B934-B06D4E490FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6BAB2C-D94B-49BC-BB65-118CB0E4A406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{84E4215D-59A1-47B3-B7C6-EBA92DED9849}"/>
   </bookViews>
@@ -240,12 +240,6 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -256,40 +250,46 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -639,127 +639,127 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="30.140625" defaultRowHeight="42" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" style="3"/>
-    <col min="3" max="3" width="30.140625" style="3" customWidth="1"/>
-    <col min="4" max="16384" width="30.140625" style="3"/>
+    <col min="1" max="1" width="30.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" style="1"/>
+    <col min="3" max="3" width="30.140625" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="30.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="H1" s="4"/>
+      <c r="F1" s="11"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9">
-        <f>IF(C3*0.2&lt;0,0,C3*0.2)</f>
-        <v>4000</v>
-      </c>
-      <c r="F2" s="9"/>
-      <c r="H2" s="10"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="10">
+        <f>ROUND(IF(C3*0.2&lt;0,0,C3*0.2),0)</f>
+        <v>3991</v>
+      </c>
+      <c r="F2" s="10"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
+      <c r="A3" s="6">
         <v>80000</v>
       </c>
-      <c r="B3" s="11">
-        <v>60000</v>
-      </c>
-      <c r="C3" s="9">
+      <c r="B3" s="6">
+        <v>60047</v>
+      </c>
+      <c r="C3" s="10">
         <f>A3-B3</f>
-        <v>20000</v>
-      </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
+        <v>19953</v>
+      </c>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="2" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="9">
-        <f>IF(C6&lt;=125000,0,(C6-125000)*0.125)</f>
+      <c r="D5" s="14"/>
+      <c r="E5" s="10">
+        <f>ROUND(IF(C6&lt;=125000,0,(C6-125000)*0.125),0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="A6" s="6">
         <v>650000</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="6">
         <v>700000</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="18">
         <f>A6-B6</f>
         <v>-50000</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="9">
+      <c r="B7" s="9"/>
+      <c r="C7" s="10">
         <f>SUM(E2,E5)</f>
-        <v>4000</v>
-      </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
+        <v>3991</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8">
         <f>C3+C6</f>
-        <v>-30000</v>
-      </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
+        <v>-30047</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>